<commit_message>
domain make it optional and if not given then make it using the school name (removing spaces) give note, incase of more than one branch, user will be able to add new branches once the account has been setup if exact begin and end dates for school year are not known can they be changed later remove back button from initial wizard, previous is enough give better password rules send link to verify email instead of dashboard take to settings directly
</commit_message>
<xml_diff>
--- a/scripts/templates/settings-onboarding-template.xlsx
+++ b/scripts/templates/settings-onboarding-template.xlsx
@@ -3,15 +3,16 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="academic_years" sheetId="1" r:id="rId1"/>
-    <sheet name="subjects" sheetId="2" r:id="rId2"/>
-    <sheet name="classes" sheetId="3" r:id="rId3"/>
-    <sheet name="sections" sheetId="4" r:id="rId4"/>
-    <sheet name="levels" sheetId="5" r:id="rId5"/>
-    <sheet name="assessment_types" sheetId="6" r:id="rId6"/>
-    <sheet name="leave_quota" sheetId="7" r:id="rId7"/>
-    <sheet name="library_categories" sheetId="8" r:id="rId8"/>
-    <sheet name="inventory_categories" sheetId="9" r:id="rId9"/>
+    <sheet name="subjects" sheetId="1" r:id="rId1"/>
+    <sheet name="classes" sheetId="2" r:id="rId2"/>
+    <sheet name="levels" sheetId="3" r:id="rId3"/>
+    <sheet name="assessment_types" sheetId="4" r:id="rId4"/>
+    <sheet name="subject_templates" sheetId="5" r:id="rId5"/>
+    <sheet name="school_days" sheetId="6" r:id="rId6"/>
+    <sheet name="timing_templates" sheetId="7" r:id="rId7"/>
+    <sheet name="timing_slots" sheetId="8" r:id="rId8"/>
+    <sheet name="grade_templates" sheetId="9" r:id="rId9"/>
+    <sheet name="grade_ranges" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -405,77 +406,559 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:C4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>name</v>
       </c>
       <c r="B1" t="str">
-        <v>start_date</v>
+        <v>code</v>
       </c>
       <c r="C1" t="str">
-        <v>end_date</v>
-      </c>
-      <c r="D1" t="str">
-        <v>set_active</v>
+        <v>lang_code</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-2027</v>
+        <v>Mathematics</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-09-01</v>
+        <v>MATH</v>
       </c>
       <c r="C2" t="str">
-        <v>2027-06-30</v>
-      </c>
-      <c r="D2" t="str">
-        <v>true</v>
+        <v>EN</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>رياضيات</v>
+      </c>
+      <c r="B3" t="str">
+        <v>MATH</v>
+      </c>
+      <c r="C3" t="str">
+        <v>AR</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>English</v>
+      </c>
+      <c r="B4" t="str">
+        <v>ENG</v>
+      </c>
+      <c r="C4" t="str">
+        <v>EN</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:E6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>name_en</v>
+        <v>template_name</v>
       </c>
       <c r="B1" t="str">
-        <v>name_ar</v>
+        <v>letter</v>
       </c>
       <c r="C1" t="str">
-        <v>code</v>
+        <v>min_percentage</v>
+      </c>
+      <c r="D1" t="str">
+        <v>max_percentage</v>
+      </c>
+      <c r="E1" t="str">
+        <v>sort_order</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Mathematics</v>
+        <v>Primary Grades</v>
       </c>
       <c r="B2" t="str">
-        <v>رياضيات</v>
+        <v>A</v>
       </c>
       <c r="C2" t="str">
-        <v>MATH</v>
+        <v>80</v>
+      </c>
+      <c r="D2" t="str">
+        <v>100</v>
+      </c>
+      <c r="E2" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Primary Grades</v>
+      </c>
+      <c r="B3" t="str">
+        <v>B</v>
+      </c>
+      <c r="C3" t="str">
+        <v>65</v>
+      </c>
+      <c r="D3" t="str">
+        <v>79</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Primary Grades</v>
+      </c>
+      <c r="B4" t="str">
+        <v>C</v>
+      </c>
+      <c r="C4" t="str">
+        <v>50</v>
+      </c>
+      <c r="D4" t="str">
+        <v>64</v>
+      </c>
+      <c r="E4" t="str">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Primary Grades</v>
+      </c>
+      <c r="B5" t="str">
+        <v>D</v>
+      </c>
+      <c r="C5" t="str">
+        <v>40</v>
+      </c>
+      <c r="D5" t="str">
+        <v>49</v>
+      </c>
+      <c r="E5" t="str">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Primary Grades</v>
+      </c>
+      <c r="B6" t="str">
+        <v>F</v>
+      </c>
+      <c r="C6" t="str">
+        <v>0</v>
+      </c>
+      <c r="D6" t="str">
+        <v>39</v>
+      </c>
+      <c r="E6" t="str">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>display_name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>sort_order</v>
+      </c>
+      <c r="D1" t="str">
+        <v>section_names</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Grade 1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Grade 1</v>
+      </c>
+      <c r="C2" t="str">
+        <v>1</v>
+      </c>
+      <c r="D2" t="str">
+        <v>A,B</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Grade 2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Grade 2</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2</v>
+      </c>
+      <c r="D3" t="str">
+        <v>A,B</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>class_names</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Primary</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Grade 1,Grade 2</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>code</v>
+      </c>
+      <c r="C1" t="str">
+        <v>lang_code</v>
+      </c>
+      <c r="D1" t="str">
+        <v>sort_order</v>
+      </c>
+      <c r="E1" t="str">
+        <v>is_term_examination</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Mid Term</v>
+      </c>
+      <c r="B2" t="str">
+        <v>MID</v>
+      </c>
+      <c r="C2" t="str">
+        <v>EN</v>
+      </c>
+      <c r="D2" t="str">
+        <v>1</v>
+      </c>
+      <c r="E2" t="str">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Final</v>
+      </c>
+      <c r="B3" t="str">
+        <v>FINAL</v>
+      </c>
+      <c r="C3" t="str">
+        <v>EN</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2</v>
+      </c>
+      <c r="E3" t="str">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Quiz</v>
+      </c>
+      <c r="B4" t="str">
+        <v>QUIZ</v>
+      </c>
+      <c r="C4" t="str">
+        <v>EN</v>
+      </c>
+      <c r="D4" t="str">
+        <v>3</v>
+      </c>
+      <c r="E4" t="str">
+        <v>no</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>description</v>
+      </c>
+      <c r="C1" t="str">
+        <v>subject_names</v>
+      </c>
+      <c r="D1" t="str">
+        <v>assign_mode</v>
+      </c>
+      <c r="E1" t="str">
+        <v>assign_names</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Primary Core</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Core subjects for primary classes</v>
+      </c>
+      <c r="C2" t="str">
+        <v>MATH,ENG</v>
+      </c>
+      <c r="D2" t="str">
+        <v>classes</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Grade 1,Grade 2</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B8"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>day</v>
+      </c>
+      <c r="B1" t="str">
+        <v>active</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Sunday</v>
+      </c>
+      <c r="B2" t="str">
+        <v>N</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Monday</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Wednesday</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Friday</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Y</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Saturday</v>
+      </c>
+      <c r="B8" t="str">
+        <v>N</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>start_time</v>
+      </c>
+      <c r="C1" t="str">
+        <v>end_time</v>
+      </c>
+      <c r="D1" t="str">
+        <v>period_duration_minutes</v>
+      </c>
+      <c r="E1" t="str">
+        <v>assigned_class_names</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Primary Day</v>
+      </c>
+      <c r="B2" t="str">
+        <v>07:30</v>
+      </c>
+      <c r="C2" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="D2" t="str">
+        <v>40</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Grade 1,Grade 2</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>template_name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>slot_name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>start_time</v>
+      </c>
+      <c r="D1" t="str">
+        <v>end_time</v>
+      </c>
+      <c r="E1" t="str">
+        <v>sort_order</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Primary Day</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Break</v>
+      </c>
+      <c r="C2" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="D2" t="str">
+        <v>10:20</v>
+      </c>
+      <c r="E2" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Primary Day</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Lunch</v>
+      </c>
+      <c r="C3" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="D3" t="str">
+        <v>12:40</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C2"/>
   <sheetData>
@@ -484,21 +967,21 @@
         <v>name</v>
       </c>
       <c r="B1" t="str">
-        <v>display_name</v>
+        <v>assigned_class_names</v>
       </c>
       <c r="C1" t="str">
-        <v>sort_order</v>
+        <v>minimum_passing_grade</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Grade 1</v>
+        <v>Primary Grades</v>
       </c>
       <c r="B2" t="str">
-        <v>Grade 1</v>
+        <v>Grade 1,Grade 2</v>
       </c>
       <c r="C2" t="str">
-        <v>1</v>
+        <v>D</v>
       </c>
     </row>
   </sheetData>
@@ -506,154 +989,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>sort_order</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>A</v>
-      </c>
-      <c r="B2" t="str">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>class_names</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Primary</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Grade 1,Grade 2,Grade 3</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>name_en</v>
-      </c>
-      <c r="B1" t="str">
-        <v>name_ar</v>
-      </c>
-      <c r="C1" t="str">
-        <v>sort_order</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Quiz</v>
-      </c>
-      <c r="B2" t="str">
-        <v>اختبار قصير</v>
-      </c>
-      <c r="C2" t="str">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>annual_quota</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>10</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>category</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>General Knowledge</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>category</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Uniforms</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A2"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>